<commit_message>
chore: resolve unmatched validations + highlight the excel file
</commit_message>
<xml_diff>
--- a/rules/CORE-000199/negative/01/data/unit-test-coreid-CG0406-negative.xlsx
+++ b/rules/CORE-000199/negative/01/data/unit-test-coreid-CG0406-negative.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,7 +577,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -590,22 +590,22 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OETEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -633,7 +633,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -646,22 +646,22 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OETEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -702,22 +702,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OETEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -745,7 +745,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -758,22 +758,22 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OETEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -801,7 +801,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -814,22 +814,22 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OETEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -857,11 +857,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>vs.xpt</t>
+          <t>oe.xpt</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -870,26 +870,26 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>VSTEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>vs.xpt</t>
+          <t>oe.xpt</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -898,26 +898,26 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>VSTEST</t>
+          <t>OETEST</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>vs.xpt</t>
+          <t>oe.xpt</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -926,26 +926,26 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>VSTEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>vs.xpt</t>
+          <t>oe.xpt</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -954,26 +954,26 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>VSTEST</t>
+          <t>OETEST</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>vs.xpt</t>
+          <t>oe.xpt</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -982,26 +982,26 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>VSTEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>vs.xpt</t>
+          <t>oe.xpt</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1010,100 +1010,660 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>VSTEST</t>
+          <t>OETEST</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>oe.xpt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>11</v>
-      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>VSTEST</t>
+          <t>OETESTCD</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+          <t>INTP</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>oe.xpt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>vs.xpt</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Record</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>12</v>
-      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>VSTEST</t>
+          <t>OETEST</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>oe.xpt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>19</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>OETESTCD</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>INTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>11</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>oe.xpt</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>OETEST</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Interpretationaaaaaaaaaaaaaaaaaaaaaaaaaadd</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>oe.xpt</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>OETESTCD</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>INTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>12</v>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>vs.xpt</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Record</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D24" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>VSTEST</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>DIABP</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
         <v>13</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>VSTEST</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>13</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>6</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>DIABP</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>14</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>7</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>VSTEST</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>14</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>7</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>DIABP</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>15</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>8</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>VSTEST</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>15</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>8</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>DIABP</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>16</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>9</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>VSTEST</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>16</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>9</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>DIABP</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>17</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>VSTEST</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>17</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>10</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>DIABP</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>18</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>11</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>VSTEST</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>18</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>11</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>DIABP</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>19</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>12</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>VSTEST</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>19</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>12</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>DIABP</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>20</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>13</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>VSTEST</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>DiastolicBloodPressureDiastolicBloodPressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>20</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>vs.xpt</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>13</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>VSTESTCD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>DIABP</t>
         </is>
       </c>
     </row>
@@ -1477,7 +2037,7 @@
       <c r="E5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -1558,7 +2118,7 @@
       <c r="E6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -1963,7 +2523,7 @@
       <c r="E11" t="n">
         <v>7</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -2049,7 +2609,7 @@
       <c r="E12" t="n">
         <v>8</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -2216,7 +2776,7 @@
       <c r="E14" t="n">
         <v>10</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -2297,7 +2857,7 @@
       <c r="E15" t="n">
         <v>11</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -2378,7 +2938,7 @@
       <c r="E16" t="n">
         <v>5</v>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -2464,7 +3024,7 @@
       <c r="E17" t="n">
         <v>6</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -2550,7 +3110,7 @@
       <c r="E18" t="n">
         <v>7</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -2631,7 +3191,7 @@
       <c r="E19" t="n">
         <v>7</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -2717,7 +3277,7 @@
       <c r="E20" t="n">
         <v>8</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>INTP</t>
         </is>
@@ -3603,7 +4163,7 @@
       <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>
@@ -3678,7 +4238,7 @@
       <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>
@@ -3753,7 +4313,7 @@
       <c r="D7" t="n">
         <v>3</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>
@@ -3833,7 +4393,7 @@
       <c r="D8" t="n">
         <v>4</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>
@@ -3908,7 +4468,7 @@
       <c r="D9" t="n">
         <v>5</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>
@@ -3983,7 +4543,7 @@
       <c r="D10" t="n">
         <v>6</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>
@@ -4061,7 +4621,7 @@
       <c r="D11" t="n">
         <v>7</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>
@@ -4139,7 +4699,7 @@
       <c r="D12" t="n">
         <v>8</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>
@@ -4217,7 +4777,7 @@
       <c r="D13" t="n">
         <v>9</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>DIABP</t>
         </is>

</xml_diff>